<commit_message>
Actualizado documento estancias formativas
</commit_message>
<xml_diff>
--- a/documentos/Estancias formativas.xlsx
+++ b/documentos/Estancias formativas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\enolc\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1BB62B34-4BEE-4378-AFA1-35490402FB30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D5F5A7A9-F44F-4C5D-846B-B922B02FB547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="35">
   <si>
     <t>Alumno/a:</t>
   </si>
@@ -74,9 +74,6 @@
     <t>Creación de 3 primeras imágenes y guiones</t>
   </si>
   <si>
-    <t>4 h productivas</t>
-  </si>
-  <si>
     <t>2 h</t>
   </si>
   <si>
@@ -87,6 +84,54 @@
   </si>
   <si>
     <t>Creación de 3 siguientes imágenes y audios</t>
+  </si>
+  <si>
+    <t>Revisión, ampliación guión Julio César</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Organización de escenas para grabación </t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 h </t>
+  </si>
+  <si>
+    <t>2 h y 30 min</t>
+  </si>
+  <si>
+    <t>Generación audios reportero y preparación</t>
+  </si>
+  <si>
+    <t>4 h y 30 min</t>
+  </si>
+  <si>
+    <t>Inicio montaje de escenas con HeyGen</t>
+  </si>
+  <si>
+    <t>Creación primer video de prueba HeyGen</t>
+  </si>
+  <si>
+    <t>Comprobación funcionamiento personajes</t>
+  </si>
+  <si>
+    <t>Ajustes posición reportero y Julio César</t>
+  </si>
+  <si>
+    <t>Pruebas para que aparezcan ambos juntos</t>
+  </si>
+  <si>
+    <t>Mejora aspecto visual reportero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisión guión para ajustar duración </t>
+  </si>
+  <si>
+    <t>Revisión general del proyecto</t>
+  </si>
+  <si>
+    <t>1 h y 30 min</t>
+  </si>
+  <si>
+    <t>Planificacón siguientes pasos proyecto</t>
   </si>
 </sst>
 </file>
@@ -999,10 +1044,10 @@
         <v>0.54166666666666663</v>
       </c>
       <c r="E8" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="8" t="s">
         <v>17</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>18</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>9</v>
@@ -1022,7 +1067,7 @@
         <v>14</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>2</v>
@@ -1039,121 +1084,301 @@
         <v>0.5625</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B11" s="11"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
+      <c r="B11" s="11">
+        <v>46125</v>
+      </c>
+      <c r="C11" s="12">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="D11" s="12">
+        <v>0.8125</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B12" s="11"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
+      <c r="B12" s="11">
+        <v>46125</v>
+      </c>
+      <c r="C12" s="12">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="D12" s="12">
+        <v>0.8125</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B13" s="11"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
+      <c r="B13" s="11">
+        <v>46126</v>
+      </c>
+      <c r="C13" s="12">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D13" s="12">
+        <v>0.60069444444444442</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B14" s="11"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
+      <c r="B14" s="11">
+        <v>46126</v>
+      </c>
+      <c r="C14" s="12">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D14" s="12">
+        <v>0.60069444444444442</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B15" s="11"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
+      <c r="B15" s="11">
+        <v>46127</v>
+      </c>
+      <c r="C15" s="12">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="D15" s="12">
+        <v>0.8125</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B16" s="11"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B17" s="11"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B18" s="11"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B19" s="11"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B20" s="11"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B21" s="11"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B22" s="11"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-    </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B16" s="11">
+        <v>46127</v>
+      </c>
+      <c r="C16" s="12">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="D16" s="12">
+        <v>0.8125</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="11">
+        <v>46128</v>
+      </c>
+      <c r="C17" s="12">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D17" s="12">
+        <v>0.60069444444444442</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="11">
+        <v>46128</v>
+      </c>
+      <c r="C18" s="12">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D18" s="12">
+        <v>0.60069444444444442</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B19" s="11">
+        <v>46129</v>
+      </c>
+      <c r="C19" s="12">
+        <v>0.75</v>
+      </c>
+      <c r="D19" s="12">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="11">
+        <v>46129</v>
+      </c>
+      <c r="C20" s="12">
+        <v>0.75</v>
+      </c>
+      <c r="D20" s="12">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B21" s="11">
+        <v>46130</v>
+      </c>
+      <c r="C21" s="12">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="D21" s="12">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="11">
+        <v>46130</v>
+      </c>
+      <c r="C22" s="12">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="D22" s="12">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="11"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12"/>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="11"/>
       <c r="C24" s="12"/>
       <c r="D24" s="12"/>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B25" s="11"/>
       <c r="C25" s="12"/>
       <c r="D25" s="12"/>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="11"/>
       <c r="C26" s="12"/>
       <c r="D26" s="12"/>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B27" s="11"/>
       <c r="C27" s="12"/>
       <c r="D27" s="12"/>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B28" s="11"/>
       <c r="C28" s="12"/>
       <c r="D28" s="12"/>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B29" s="11"/>
       <c r="C29" s="12"/>
       <c r="D29" s="12"/>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B30" s="11"/>
       <c r="C30" s="12"/>
       <c r="D30" s="12"/>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="11"/>
       <c r="C31" s="12"/>
       <c r="D31" s="12"/>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="11"/>
       <c r="C32" s="12"/>
       <c r="D32" s="12"/>
@@ -1896,23 +2121,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="e90a08e0-bb8b-401b-a3a3-8c2e123990c6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007CE3C27FCDB74D4C843739AA6B24DB49" ma:contentTypeVersion="18" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="9ddedeecd07a3c7537ac720e3c1040bf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="e9628731-4a47-4a59-8d6b-c3de1e8c280e" xmlns:ns4="e90a08e0-bb8b-401b-a3a3-8c2e123990c6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e6cadf8ef5868d961660339076726392" ns3:_="" ns4:_="">
     <xsd:import namespace="e9628731-4a47-4a59-8d6b-c3de1e8c280e"/>
@@ -2165,32 +2373,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0267A2D9-87B5-4FAB-A4C3-E17C5A6D49AE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="e90a08e0-bb8b-401b-a3a3-8c2e123990c6"/>
-    <ds:schemaRef ds:uri="e9628731-4a47-4a59-8d6b-c3de1e8c280e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3AA5E020-D143-490C-9C50-B50AB0A29557}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="e90a08e0-bb8b-401b-a3a3-8c2e123990c6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4EC3E362-CE68-4F90-B331-45D93B7D65C2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2207,4 +2407,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3AA5E020-D143-490C-9C50-B50AB0A29557}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0267A2D9-87B5-4FAB-A4C3-E17C5A6D49AE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e90a08e0-bb8b-401b-a3a3-8c2e123990c6"/>
+    <ds:schemaRef ds:uri="e9628731-4a47-4a59-8d6b-c3de1e8c280e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>